<commit_message>
Cambia COSTO_LD_SF basados en enero 2025
</commit_message>
<xml_diff>
--- a/DATASOURCE.xlsx
+++ b/DATASOURCE.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30125"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{EAE0BDB8-E038-45D2-B8B8-E62FBBC35DBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{3B59E5F3-156E-4E00-881B-82CC51C71E19}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="5" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SETS" sheetId="1" r:id="rId1"/>
@@ -56,7 +56,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="429" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="431" uniqueCount="53">
   <si>
     <t>PLANTA</t>
   </si>
@@ -146,6 +146,12 @@
   </si>
   <si>
     <t>COSTO_LD_SF</t>
+  </si>
+  <si>
+    <t>38.61</t>
+  </si>
+  <si>
+    <t>34.75</t>
   </si>
   <si>
     <t>COSTO</t>
@@ -523,7 +529,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyBorder="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
@@ -577,12 +583,18 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="4" fontId="0" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="4" fontId="0" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1287,40 +1299,42 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:K6"/>
   <sheetFormatPr defaultColWidth="10.5703125" defaultRowHeight="13.9"/>
   <cols>
-    <col min="2" max="2" width="22.7109375" customWidth="1"/>
+    <col min="1" max="1" width="10.5703125" style="44"/>
+    <col min="2" max="2" width="22.7109375" style="44" customWidth="1"/>
     <col min="3" max="3" width="13.140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" s="27" t="s">
+      <c r="A1" s="43" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="27" t="s">
+      <c r="B1" s="43" t="s">
         <v>29</v>
       </c>
       <c r="K1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:11">
-      <c r="A2" s="27" t="s">
+    <row r="2" spans="1:11" ht="15">
+      <c r="A2" s="43" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="27">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11">
-      <c r="A3" s="27" t="s">
+      <c r="B2" s="43" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" ht="15">
+      <c r="A3" s="43" t="s">
         <v>9</v>
       </c>
-      <c r="B3" s="27">
-        <v>18</v>
-      </c>
-    </row>
+      <c r="B3" s="43" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" ht="15"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -1351,16 +1365,16 @@
         <v>1</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="G1" s="27" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="H1" s="27" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="I1" s="27" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="2" spans="1:9">
@@ -3690,15 +3704,15 @@
         <v>26</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="F1" s="39" t="s">
-        <v>36</v>
-      </c>
-      <c r="G1" s="39"/>
+        <v>37</v>
+      </c>
+      <c r="F1" s="42" t="s">
+        <v>38</v>
+      </c>
+      <c r="G1" s="42"/>
     </row>
     <row r="2" spans="1:12">
       <c r="A2" s="5" t="s">
@@ -3712,7 +3726,7 @@
         <v>802978.3523250001</v>
       </c>
       <c r="F2" s="18" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="G2" s="19">
         <v>0.03</v>
@@ -3730,7 +3744,7 @@
         <v>446099.08462500002</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="G3" s="19">
         <v>0.45</v>
@@ -3748,12 +3762,12 @@
         <v>321191.34093000001</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="G4" s="19">
         <v>0.25</v>
       </c>
-      <c r="K4" s="42"/>
+      <c r="K4" s="41"/>
     </row>
     <row r="5" spans="1:12">
       <c r="A5" s="9" t="s">
@@ -3767,12 +3781,12 @@
         <v>214127.56062</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="G5" s="19">
         <v>0.18</v>
       </c>
-      <c r="K5" s="42"/>
+      <c r="K5" s="41"/>
       <c r="L5" s="12"/>
     </row>
     <row r="6" spans="1:12">
@@ -3787,12 +3801,12 @@
         <v>465349.48267499992</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="G6" s="19">
         <v>0.12</v>
       </c>
-      <c r="K6" s="42"/>
+      <c r="K6" s="41"/>
     </row>
     <row r="7" spans="1:12">
       <c r="A7" s="7" t="s">
@@ -3805,7 +3819,7 @@
         <f>$G10*$G$2*$G4</f>
         <v>258527.49037499996</v>
       </c>
-      <c r="K7" s="42"/>
+      <c r="K7" s="41"/>
     </row>
     <row r="8" spans="1:12">
       <c r="A8" s="7" t="s">
@@ -3819,12 +3833,12 @@
         <v>186139.79306999996</v>
       </c>
       <c r="F8" s="22" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="G8" s="23" t="s">
-        <v>43</v>
-      </c>
-      <c r="K8" s="42"/>
+        <v>45</v>
+      </c>
+      <c r="K8" s="41"/>
     </row>
     <row r="9" spans="1:12">
       <c r="A9" s="9" t="s">
@@ -3838,13 +3852,13 @@
         <v>124093.19537999998</v>
       </c>
       <c r="F9" s="36" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="G9" s="37">
         <v>59479877.950000003</v>
       </c>
       <c r="I9" s="24"/>
-      <c r="K9" s="42"/>
+      <c r="K9" s="41"/>
     </row>
     <row r="10" spans="1:12">
       <c r="A10" s="5" t="s">
@@ -3858,13 +3872,13 @@
         <v>59666.039869499997</v>
       </c>
       <c r="F10" s="36" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="G10" s="37">
         <v>34470332.049999997</v>
       </c>
       <c r="I10" s="24"/>
-      <c r="K10" s="42"/>
+      <c r="K10" s="41"/>
     </row>
     <row r="11" spans="1:12">
       <c r="A11" s="7" t="s">
@@ -3878,13 +3892,13 @@
         <v>33147.799927499997</v>
       </c>
       <c r="F11" s="36" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="G11" s="37">
         <v>4419706.6569999997</v>
       </c>
-      <c r="K11" s="42"/>
-      <c r="L11" s="42"/>
+      <c r="K11" s="41"/>
+      <c r="L11" s="41"/>
     </row>
     <row r="12" spans="1:12" ht="13.5" customHeight="1">
       <c r="A12" s="7" t="s">
@@ -3898,7 +3912,7 @@
         <v>23866.415947799997</v>
       </c>
       <c r="F12" s="36" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="G12" s="37">
         <v>1009270</v>
@@ -3952,7 +3966,7 @@
         <v>7569.5249999999996</v>
       </c>
       <c r="F15" s="38" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="G15" s="37">
         <v>16191735</v>
@@ -3970,7 +3984,7 @@
         <v>5450.0579999999991</v>
       </c>
       <c r="F16" s="36" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="G16" s="37">
         <v>5209870</v>
@@ -4094,7 +4108,7 @@
       <c r="B26" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="C26" s="41">
+      <c r="C26" s="40">
         <f>$G$15*$G$2*$G3</f>
         <v>218588.42249999999</v>
       </c>
@@ -4118,7 +4132,7 @@
       <c r="B28" t="s">
         <v>13</v>
       </c>
-      <c r="C28" s="40">
+      <c r="C28" s="39">
         <f>$G$15*$G$2*$G5</f>
         <v>87435.368999999992</v>
       </c>
@@ -4202,7 +4216,7 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" s="25" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="2" spans="1:1">

</xml_diff>